<commit_message>
Daily EOD data and reports for 2026-08-05
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260805.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260805.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.332</v>
+        <v>1.415</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.012</v>
+        <v>0.095</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.91%</t>
+          <t>7.20%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>204037.09</v>
+        <v>216751.12</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>1838.17</v>
+        <v>14552.19</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.19</v>
+        <v>2.18</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.39%</t>
+          <t>0.93%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>153300</v>
+        <v>152600</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>2100</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1.095</v>
+        <v>1.1</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.055</v>
+        <v>0.06</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>5.29%</t>
+          <t>5.77%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>57458</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>62916.51</v>
+        <v>63203.8</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>3160.19</v>
+        <v>3447.48</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>62.08</v>
+        <v>62.54</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>1.56</v>
+        <v>2.02</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.58%</t>
+          <t>3.34%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>686915.2</v>
+        <v>692005.1</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>17261.4</v>
+        <v>22351.3</v>
       </c>
     </row>
     <row r="8">
@@ -596,24 +596,24 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-0.003</v>
+        <v>0</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
         <v>44090</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0</v>
+        <v>132.27</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-132.27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>179.71</v>
+        <v>178.23</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-1.01</v>
+        <v>-2.49</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.56%</t>
+          <t>-1.38%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.782</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.017</v>
+        <v>0.05</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.22%</t>
+          <t>6.54%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>7820</v>
+        <v>8150</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>170</v>
+        <v>500</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>130.08</v>
+        <v>130.66</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>1.25</v>
+        <v>1.83</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.97%</t>
+          <t>1.42%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>520320</v>
+        <v>522640</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>5000</v>
+        <v>7320</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0</v>
+        <v>0.27</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-0.275</v>
+        <v>-0.005</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>-1.82%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>0</v>
+        <v>5400</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>-5500</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="13">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.093</v>
+        <v>0.091</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.005</v>
+        <v>0.003</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>5.68%</t>
+          <t>3.41%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>875.3200000000001</v>
+        <v>856.49</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>47.06</v>
+        <v>28.24</v>
       </c>
     </row>
     <row r="15">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>0.105</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.105</v>
+        <v>0</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>630</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-630</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>38.87</v>
+        <v>38.53</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.05</v>
+        <v>-0.29</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.13%</t>
+          <t>-0.75%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>32.07</v>
+        <v>31.78</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-0.88</v>
+        <v>-1.17</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-2.67%</t>
+          <t>-3.55%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>41306.16</v>
+        <v>40932.64</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-1133.44</v>
+        <v>-1506.96</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1677490.28</v>
+        <v>1703301.42</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>20781.11</v>
+        <v>46592.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>